<commit_message>
Publish Duisburg_2023_WCH, Szeged_2023_WC, Vejen_2023_MAR
</commit_message>
<xml_diff>
--- a/events/Vejen_2023_MAR/Vejen_2023_MAR_Results.xlsx
+++ b/events/Vejen_2023_MAR/Vejen_2023_MAR_Results.xlsx
@@ -3695,6 +3695,11 @@
           <t>00:16:53.640</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9728,6 +9733,11 @@
       <c r="P141" t="inlineStr">
         <is>
           <t>00:16:26.420</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>47779</t>
         </is>
       </c>
     </row>
@@ -29499,7 +29509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D306"/>
+  <dimension ref="A1:D307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36234,6 +36244,28 @@
         </is>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>BEDEC</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>